<commit_message>
Update AI summary pipeline with improved comparison periods, adjusted word limit handling, and HAI calculation fixes
</commit_message>
<xml_diff>
--- a/Metric Topics (DRAFT).xlsx
+++ b/Metric Topics (DRAFT).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tipstrategiesinc-my.sharepoint.com/personal/tip_theoryintopractice_com/Documents/ANALYSIS/DELIVERABLE TOOLS - Tableau/_dashboards/Baseline/components/AI Summary/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="557" documentId="8_{B343592D-7386-44F8-9DBC-D05530D49B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{57E0F837-5DE1-4B2D-929C-D967EA83D8BF}"/>
+  <xr:revisionPtr revIDLastSave="558" documentId="8_{B343592D-7386-44F8-9DBC-D05530D49B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F84A6574-AAB2-4309-8F0F-1DB7F35BBF00}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{4F89DE8C-5445-44C5-A37C-A3AFB7DF52A1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{4F89DE8C-5445-44C5-A37C-A3AFB7DF52A1}"/>
   </bookViews>
   <sheets>
     <sheet name="v1" sheetId="2" r:id="rId1"/>
@@ -57,18 +57,21 @@
     </comment>
     <comment ref="H60" authorId="1" shapeId="0" xr:uid="{01FA5E3D-28A7-49CC-8C95-B5794847581E}">
       <text>
-        <t>[Threaded comment]
+        <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    HAI calculated using standard assumptions of 20% down payment at 30 years with a 0.2 qualifying ratio is calculated as:
+    HAI calculated using standard assumptions of 20% down payment at 30 years with a 0.2 qualifying ratio is calculated as (corrected 7/22):
+(Median HH Income)/
+{
 [
-(Median HH Income)/
 ((Avg. 30-year rate)/12)*(0.8)*(Median List Price)
 ]
 /
 [
-(1-(1+((Avg. 30-year rate)/12)^((-12)*30) ))*(12/0.2)
-]</t>
+1-(1+((Avg. 30-year rate)/12)^((-12)*30) )
+] 
+} * (12/0.2)
+</t>
       </text>
     </comment>
   </commentList>
@@ -781,10 +784,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
@@ -798,7 +800,7 @@
     <dxf>
       <border outline="0">
         <bottom style="thin">
-          <color rgb="FF000000"/>
+          <color indexed="64"/>
         </bottom>
       </border>
     </dxf>
@@ -825,7 +827,7 @@
     <dxf>
       <border outline="0">
         <bottom style="thin">
-          <color indexed="64"/>
+          <color rgb="FF000000"/>
         </bottom>
       </border>
     </dxf>
@@ -893,14 +895,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C80B2413-554A-4D18-A78D-6C8F504015B1}" name="Table13" displayName="Table13" ref="A1:M27" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{C80B2413-554A-4D18-A78D-6C8F504015B1}" name="Table13" displayName="Table13" ref="A1:M27" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
   <autoFilter ref="A1:M27" xr:uid="{F041D1FB-A3F2-4260-B8C6-424FC0E756D1}"/>
   <tableColumns count="13">
     <tableColumn id="13" xr3:uid="{949BC6E5-3D05-4A6C-94C2-CB908ABDA89A}" name="Topic"/>
     <tableColumn id="1" xr3:uid="{B733B87F-BC8C-4D6F-B28D-031628E6B4E5}" name="Comparison Period"/>
     <tableColumn id="2" xr3:uid="{B54F27B9-6AC5-457D-B474-54CA76C97A0C}" name="Current Period"/>
     <tableColumn id="3" xr3:uid="{3DE3AEF6-C81A-4612-AFC0-D9F1C29FAE98}" name="Data Source"/>
-    <tableColumn id="4" xr3:uid="{0B2615BE-D5DD-4845-B905-64571944806D}" name="Variables" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{0B2615BE-D5DD-4845-B905-64571944806D}" name="Variables" dataDxfId="3"/>
     <tableColumn id="5" xr3:uid="{C7141793-B437-4514-8395-367DD2C50EFC}" name="Metric"/>
     <tableColumn id="12" xr3:uid="{7EC7CF40-AC09-4F6D-A0D5-922FB3882109}" name="Metric Type"/>
     <tableColumn id="6" xr3:uid="{FA067A27-7E9B-42A4-AED7-FB549408B76B}" name="Description"/>
@@ -915,14 +917,14 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F041D1FB-A3F2-4260-B8C6-424FC0E756D1}" name="Table1" displayName="Table1" ref="A1:N45" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F041D1FB-A3F2-4260-B8C6-424FC0E756D1}" name="Table1" displayName="Table1" ref="A1:N45" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1">
   <autoFilter ref="A1:N45" xr:uid="{F041D1FB-A3F2-4260-B8C6-424FC0E756D1}"/>
   <tableColumns count="14">
     <tableColumn id="13" xr3:uid="{A7003B1A-D9ED-4F5D-BFF6-7FC58B05A484}" name="Topic"/>
     <tableColumn id="1" xr3:uid="{F89CAD15-00F2-426B-BFF5-A4D1FB9C0C54}" name="Comparison Period"/>
     <tableColumn id="2" xr3:uid="{0EF05096-32D4-4CAA-B154-CA463441DB61}" name="Current Period"/>
     <tableColumn id="3" xr3:uid="{1DE9F036-FF07-4A7D-BDE2-25F598E39C58}" name="Data Source"/>
-    <tableColumn id="4" xr3:uid="{B43EF147-9261-47C5-98FD-59ACEBC076D3}" name="Variables" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{B43EF147-9261-47C5-98FD-59ACEBC076D3}" name="Variables" dataDxfId="0"/>
     <tableColumn id="5" xr3:uid="{53A56733-A7B2-4F96-907F-4AF12B07EDB2}" name="Metric"/>
     <tableColumn id="12" xr3:uid="{D9C9791E-2A07-4135-8BD4-54545C6BE160}" name="Metric Type"/>
     <tableColumn id="6" xr3:uid="{ABE164A8-C391-46ED-B48B-3CD1CAB82BA3}" name="Description"/>
@@ -938,14 +940,14 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{73662357-B125-4414-A24C-0D1BC6883266}" name="Table14" displayName="Table14" ref="A1:N61" totalsRowShown="0" headerRowDxfId="2" headerRowBorderDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{73662357-B125-4414-A24C-0D1BC6883266}" name="Table14" displayName="Table14" ref="A1:N61" totalsRowShown="0" headerRowDxfId="8" headerRowBorderDxfId="7">
   <autoFilter ref="A1:N61" xr:uid="{F041D1FB-A3F2-4260-B8C6-424FC0E756D1}"/>
   <tableColumns count="14">
     <tableColumn id="13" xr3:uid="{232253A6-B448-43FF-819E-F60F5724866B}" name="Topic"/>
     <tableColumn id="1" xr3:uid="{47FDFD65-48FF-423F-A9EC-D6E27B7B0C3A}" name="Comparison Period"/>
     <tableColumn id="2" xr3:uid="{726A348D-1468-47E2-BBDB-9E720DE08AC3}" name="Current Period"/>
     <tableColumn id="3" xr3:uid="{BE674323-6967-4A99-8C3E-5BDFEEE70662}" name="Data Source"/>
-    <tableColumn id="4" xr3:uid="{72EADF76-D22F-40C9-BDB7-A3445193019C}" name="Variables" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{72EADF76-D22F-40C9-BDB7-A3445193019C}" name="Variables" dataDxfId="6"/>
     <tableColumn id="5" xr3:uid="{EE26800C-6CDE-4BEF-841A-0C4977355F2A}" name="Metric"/>
     <tableColumn id="12" xr3:uid="{87DA4B98-0090-4CEA-8508-0757B7504100}" name="Metric Type"/>
     <tableColumn id="6" xr3:uid="{726A7668-D4F4-4A01-85DF-DF5FF8A1FE85}" name="Description"/>
@@ -1170,40 +1172,43 @@
 (1-(1+((Avg. 30-year rate)/12)^((-12)*30) ))</text>
   </threadedComment>
   <threadedComment ref="H60" dT="2026-07-08T20:39:47.55" personId="{BD0C8C44-C4AD-48D4-9322-93A1CCEBB0F4}" id="{01FA5E3D-28A7-49CC-8C95-B5794847581E}">
-    <text>HAI calculated using standard assumptions of 20% down payment at 30 years with a 0.2 qualifying ratio is calculated as:
+    <text xml:space="preserve">HAI calculated using standard assumptions of 20% down payment at 30 years with a 0.2 qualifying ratio is calculated as (corrected 7/22):
+(Median HH Income)/
+{
 [
-(Median HH Income)/
 ((Avg. 30-year rate)/12)*(0.8)*(Median List Price)
 ]
 /
 [
-(1-(1+((Avg. 30-year rate)/12)^((-12)*30) ))*(12/0.2)
-]</text>
+1-(1+((Avg. 30-year rate)/12)^((-12)*30) )
+] 
+} * (12/0.2)
+</text>
   </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FFF6426F-6408-4DAD-A575-E47E673E7F33}">
-  <dimension ref="A1:M79"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:M27"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="88" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="67.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="115.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="50.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="56.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="51.109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="31.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="67.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="115.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="50.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="56.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="51.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="31.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
@@ -1244,7 +1249,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>65</v>
       </c>
@@ -1257,7 +1262,7 @@
       <c r="D2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" t="s">
         <v>20</v>
       </c>
       <c r="F2" t="s">
@@ -1285,7 +1290,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>65</v>
       </c>
@@ -1298,7 +1303,7 @@
       <c r="D3" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" t="s">
         <v>20</v>
       </c>
       <c r="F3" t="s">
@@ -1326,7 +1331,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>65</v>
       </c>
@@ -1367,7 +1372,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>72</v>
       </c>
@@ -1380,7 +1385,7 @@
       <c r="D5" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" t="s">
         <v>21</v>
       </c>
       <c r="F5" t="s">
@@ -1408,7 +1413,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>72</v>
       </c>
@@ -1421,7 +1426,7 @@
       <c r="D6" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" t="s">
         <v>21</v>
       </c>
       <c r="F6" t="s">
@@ -1449,7 +1454,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>72</v>
       </c>
@@ -1462,7 +1467,7 @@
       <c r="D7" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" t="s">
         <v>21</v>
       </c>
       <c r="F7" t="s">
@@ -1490,7 +1495,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>73</v>
       </c>
@@ -1503,7 +1508,7 @@
       <c r="D8" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" t="s">
         <v>22</v>
       </c>
       <c r="F8" t="s">
@@ -1531,7 +1536,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>73</v>
       </c>
@@ -1544,7 +1549,7 @@
       <c r="D9" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" t="s">
         <v>22</v>
       </c>
       <c r="F9" t="s">
@@ -1572,7 +1577,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>73</v>
       </c>
@@ -1585,7 +1590,7 @@
       <c r="D10" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" t="s">
         <v>23</v>
       </c>
       <c r="F10" t="s">
@@ -1613,7 +1618,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>73</v>
       </c>
@@ -1626,7 +1631,7 @@
       <c r="D11" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" t="s">
         <v>23</v>
       </c>
       <c r="F11" t="s">
@@ -1654,7 +1659,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>73</v>
       </c>
@@ -1667,7 +1672,7 @@
       <c r="D12" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" t="s">
         <v>24</v>
       </c>
       <c r="F12" t="s">
@@ -1695,7 +1700,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>73</v>
       </c>
@@ -1708,7 +1713,7 @@
       <c r="D13" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" t="s">
         <v>24</v>
       </c>
       <c r="F13" t="s">
@@ -1736,7 +1741,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>74</v>
       </c>
@@ -1749,7 +1754,7 @@
       <c r="D14" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" t="s">
         <v>25</v>
       </c>
       <c r="F14" t="s">
@@ -1777,7 +1782,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>74</v>
       </c>
@@ -1790,7 +1795,7 @@
       <c r="D15" t="s">
         <v>19</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" t="s">
         <v>25</v>
       </c>
       <c r="F15" t="s">
@@ -1818,7 +1823,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>76</v>
       </c>
@@ -1831,7 +1836,7 @@
       <c r="D16" t="s">
         <v>19</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" t="s">
         <v>29</v>
       </c>
       <c r="F16" t="s">
@@ -1859,7 +1864,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>76</v>
       </c>
@@ -1872,7 +1877,7 @@
       <c r="D17" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" t="s">
         <v>29</v>
       </c>
       <c r="F17" t="s">
@@ -1900,7 +1905,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>76</v>
       </c>
@@ -1913,7 +1918,7 @@
       <c r="D18" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" t="s">
         <v>31</v>
       </c>
       <c r="F18" t="s">
@@ -1941,7 +1946,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>76</v>
       </c>
@@ -1954,7 +1959,7 @@
       <c r="D19" t="s">
         <v>19</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" t="s">
         <v>31</v>
       </c>
       <c r="F19" t="s">
@@ -1982,7 +1987,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>74</v>
       </c>
@@ -1995,7 +2000,7 @@
       <c r="D20" t="s">
         <v>19</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" t="s">
         <v>34</v>
       </c>
       <c r="F20" t="s">
@@ -2023,7 +2028,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>74</v>
       </c>
@@ -2036,7 +2041,7 @@
       <c r="D21" t="s">
         <v>19</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" t="s">
         <v>34</v>
       </c>
       <c r="F21" t="s">
@@ -2064,7 +2069,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>74</v>
       </c>
@@ -2077,7 +2082,7 @@
       <c r="D22" t="s">
         <v>19</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" t="s">
         <v>37</v>
       </c>
       <c r="F22" t="s">
@@ -2105,7 +2110,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -2118,7 +2123,7 @@
       <c r="D23" t="s">
         <v>19</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="E23" t="s">
         <v>37</v>
       </c>
       <c r="F23" t="s">
@@ -2146,7 +2151,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>75</v>
       </c>
@@ -2159,7 +2164,7 @@
       <c r="D24" t="s">
         <v>19</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="E24" t="s">
         <v>38</v>
       </c>
       <c r="F24" t="s">
@@ -2187,7 +2192,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>75</v>
       </c>
@@ -2200,7 +2205,7 @@
       <c r="D25" t="s">
         <v>19</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="E25" t="s">
         <v>38</v>
       </c>
       <c r="F25" t="s">
@@ -2228,7 +2233,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>75</v>
       </c>
@@ -2241,7 +2246,7 @@
       <c r="D26" t="s">
         <v>19</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" t="s">
         <v>39</v>
       </c>
       <c r="F26" t="s">
@@ -2269,7 +2274,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>75</v>
       </c>
@@ -2282,7 +2287,7 @@
       <c r="D27" t="s">
         <v>19</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" t="s">
         <v>39</v>
       </c>
       <c r="F27" t="s">
@@ -2309,150 +2314,6 @@
       <c r="M27" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="D28" s="2"/>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="D31" s="2"/>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="D32" s="2"/>
-    </row>
-    <row r="33" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D33" s="2"/>
-    </row>
-    <row r="34" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D34" s="2"/>
-    </row>
-    <row r="35" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D35" s="2"/>
-    </row>
-    <row r="36" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D36" s="2"/>
-    </row>
-    <row r="37" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D37" s="2"/>
-    </row>
-    <row r="38" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D38" s="2"/>
-    </row>
-    <row r="39" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D39" s="2"/>
-    </row>
-    <row r="40" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D40" s="2"/>
-    </row>
-    <row r="41" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D41" s="2"/>
-    </row>
-    <row r="42" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D42" s="2"/>
-    </row>
-    <row r="43" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D43" s="2"/>
-    </row>
-    <row r="44" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D44" s="2"/>
-    </row>
-    <row r="45" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D45" s="2"/>
-    </row>
-    <row r="46" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D46" s="2"/>
-    </row>
-    <row r="47" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D47" s="2"/>
-    </row>
-    <row r="48" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D48" s="2"/>
-    </row>
-    <row r="49" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D49" s="2"/>
-    </row>
-    <row r="50" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D50" s="2"/>
-    </row>
-    <row r="51" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D51" s="2"/>
-    </row>
-    <row r="52" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D52" s="2"/>
-    </row>
-    <row r="53" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D53" s="2"/>
-    </row>
-    <row r="54" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D54" s="2"/>
-    </row>
-    <row r="57" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D57" s="2"/>
-    </row>
-    <row r="58" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D58" s="2"/>
-    </row>
-    <row r="59" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D59" s="2"/>
-    </row>
-    <row r="60" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D60" s="2"/>
-    </row>
-    <row r="61" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D61" s="2"/>
-    </row>
-    <row r="62" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D62" s="2"/>
-    </row>
-    <row r="63" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D63" s="2"/>
-    </row>
-    <row r="64" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D64" s="2"/>
-    </row>
-    <row r="65" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D65" s="2"/>
-    </row>
-    <row r="66" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D66" s="2"/>
-    </row>
-    <row r="67" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D67" s="2"/>
-    </row>
-    <row r="68" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D68" s="2"/>
-    </row>
-    <row r="69" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D69" s="2"/>
-    </row>
-    <row r="70" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D70" s="2"/>
-    </row>
-    <row r="71" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D71" s="2"/>
-    </row>
-    <row r="72" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D72" s="2"/>
-    </row>
-    <row r="73" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D73" s="2"/>
-    </row>
-    <row r="74" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D74" s="2"/>
-    </row>
-    <row r="75" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D75" s="2"/>
-    </row>
-    <row r="76" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D76" s="2"/>
-    </row>
-    <row r="77" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D77" s="2"/>
-    </row>
-    <row r="78" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D78" s="2"/>
-    </row>
-    <row r="79" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D79" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2464,25 +2325,25 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AA7646E-3F6C-41BF-BC33-2448E647855F}">
-  <dimension ref="A1:N97"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:N45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="88" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="67.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="115.33203125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="50.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="56.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="51.109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="31.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="67.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="115.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="50.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="56.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="51.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="31.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
@@ -2526,7 +2387,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>65</v>
       </c>
@@ -2539,7 +2400,7 @@
       <c r="D2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" t="s">
         <v>20</v>
       </c>
       <c r="F2" t="s">
@@ -2570,7 +2431,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>65</v>
       </c>
@@ -2583,7 +2444,7 @@
       <c r="D3" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" t="s">
         <v>20</v>
       </c>
       <c r="F3" t="s">
@@ -2614,7 +2475,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>65</v>
       </c>
@@ -2658,7 +2519,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>65</v>
       </c>
@@ -2671,7 +2532,7 @@
       <c r="D5" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" t="s">
         <v>21</v>
       </c>
       <c r="F5" t="s">
@@ -2702,7 +2563,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>65</v>
       </c>
@@ -2715,7 +2576,7 @@
       <c r="D6" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" t="s">
         <v>21</v>
       </c>
       <c r="F6" t="s">
@@ -2746,7 +2607,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>65</v>
       </c>
@@ -2759,7 +2620,7 @@
       <c r="D7" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" t="s">
         <v>21</v>
       </c>
       <c r="F7" t="s">
@@ -2790,7 +2651,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>73</v>
       </c>
@@ -2803,7 +2664,7 @@
       <c r="D8" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" t="s">
         <v>22</v>
       </c>
       <c r="F8" t="s">
@@ -2834,7 +2695,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>73</v>
       </c>
@@ -2847,7 +2708,7 @@
       <c r="D9" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" t="s">
         <v>22</v>
       </c>
       <c r="F9" t="s">
@@ -2878,7 +2739,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>73</v>
       </c>
@@ -2891,7 +2752,7 @@
       <c r="D10" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" t="s">
         <v>23</v>
       </c>
       <c r="F10" t="s">
@@ -2922,7 +2783,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>73</v>
       </c>
@@ -2935,7 +2796,7 @@
       <c r="D11" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" t="s">
         <v>23</v>
       </c>
       <c r="F11" t="s">
@@ -2966,7 +2827,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>73</v>
       </c>
@@ -2979,7 +2840,7 @@
       <c r="D12" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" t="s">
         <v>81</v>
       </c>
       <c r="F12" t="s">
@@ -3010,7 +2871,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>73</v>
       </c>
@@ -3023,7 +2884,7 @@
       <c r="D13" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" t="s">
         <v>81</v>
       </c>
       <c r="F13" t="s">
@@ -3054,7 +2915,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>73</v>
       </c>
@@ -3067,7 +2928,7 @@
       <c r="D14" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" t="s">
         <v>88</v>
       </c>
       <c r="F14" t="s">
@@ -3098,7 +2959,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>73</v>
       </c>
@@ -3111,7 +2972,7 @@
       <c r="D15" t="s">
         <v>19</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" t="s">
         <v>88</v>
       </c>
       <c r="F15" t="s">
@@ -3142,7 +3003,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>73</v>
       </c>
@@ -3155,7 +3016,7 @@
       <c r="D16" t="s">
         <v>19</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" t="s">
         <v>85</v>
       </c>
       <c r="F16" t="s">
@@ -3186,7 +3047,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>73</v>
       </c>
@@ -3199,7 +3060,7 @@
       <c r="D17" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" t="s">
         <v>85</v>
       </c>
       <c r="F17" t="s">
@@ -3230,7 +3091,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>73</v>
       </c>
@@ -3243,7 +3104,7 @@
       <c r="D18" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" t="s">
         <v>24</v>
       </c>
       <c r="F18" t="s">
@@ -3274,7 +3135,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>73</v>
       </c>
@@ -3287,7 +3148,7 @@
       <c r="D19" t="s">
         <v>19</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" t="s">
         <v>24</v>
       </c>
       <c r="F19" t="s">
@@ -3318,7 +3179,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>74</v>
       </c>
@@ -3331,7 +3192,7 @@
       <c r="D20" t="s">
         <v>19</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" t="s">
         <v>25</v>
       </c>
       <c r="F20" t="s">
@@ -3362,7 +3223,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>74</v>
       </c>
@@ -3375,7 +3236,7 @@
       <c r="D21" t="s">
         <v>19</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" t="s">
         <v>25</v>
       </c>
       <c r="F21" t="s">
@@ -3406,7 +3267,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>76</v>
       </c>
@@ -3419,7 +3280,7 @@
       <c r="D22" t="s">
         <v>19</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" t="s">
         <v>29</v>
       </c>
       <c r="F22" t="s">
@@ -3450,7 +3311,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>76</v>
       </c>
@@ -3463,7 +3324,7 @@
       <c r="D23" t="s">
         <v>19</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="E23" t="s">
         <v>29</v>
       </c>
       <c r="F23" t="s">
@@ -3494,7 +3355,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>76</v>
       </c>
@@ -3507,7 +3368,7 @@
       <c r="D24" t="s">
         <v>19</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="E24" t="s">
         <v>31</v>
       </c>
       <c r="F24" t="s">
@@ -3538,7 +3399,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>76</v>
       </c>
@@ -3551,7 +3412,7 @@
       <c r="D25" t="s">
         <v>19</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="E25" t="s">
         <v>31</v>
       </c>
       <c r="F25" t="s">
@@ -3582,7 +3443,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>76</v>
       </c>
@@ -3595,7 +3456,7 @@
       <c r="D26" t="s">
         <v>19</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" t="s">
         <v>102</v>
       </c>
       <c r="F26" t="s">
@@ -3626,7 +3487,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>76</v>
       </c>
@@ -3639,7 +3500,7 @@
       <c r="D27" t="s">
         <v>19</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" t="s">
         <v>102</v>
       </c>
       <c r="F27" t="s">
@@ -3670,7 +3531,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>76</v>
       </c>
@@ -3683,7 +3544,7 @@
       <c r="D28" t="s">
         <v>19</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E28" t="s">
         <v>105</v>
       </c>
       <c r="F28" t="s">
@@ -3714,7 +3575,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>76</v>
       </c>
@@ -3727,7 +3588,7 @@
       <c r="D29" t="s">
         <v>19</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="E29" t="s">
         <v>105</v>
       </c>
       <c r="F29" t="s">
@@ -3758,7 +3619,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>76</v>
       </c>
@@ -3771,7 +3632,7 @@
       <c r="D30" t="s">
         <v>19</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="E30" t="s">
         <v>108</v>
       </c>
       <c r="F30" t="s">
@@ -3802,7 +3663,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>76</v>
       </c>
@@ -3815,7 +3676,7 @@
       <c r="D31" t="s">
         <v>19</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="E31" t="s">
         <v>108</v>
       </c>
       <c r="F31" t="s">
@@ -3846,7 +3707,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>74</v>
       </c>
@@ -3859,7 +3720,7 @@
       <c r="D32" t="s">
         <v>19</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="E32" t="s">
         <v>34</v>
       </c>
       <c r="F32" t="s">
@@ -3890,7 +3751,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>74</v>
       </c>
@@ -3903,7 +3764,7 @@
       <c r="D33" t="s">
         <v>19</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="E33" t="s">
         <v>34</v>
       </c>
       <c r="F33" t="s">
@@ -3934,7 +3795,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>74</v>
       </c>
@@ -3947,7 +3808,7 @@
       <c r="D34" t="s">
         <v>19</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="E34" t="s">
         <v>93</v>
       </c>
       <c r="F34" t="s">
@@ -3978,7 +3839,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>74</v>
       </c>
@@ -3991,7 +3852,7 @@
       <c r="D35" t="s">
         <v>19</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="E35" t="s">
         <v>93</v>
       </c>
       <c r="F35" t="s">
@@ -4022,7 +3883,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>74</v>
       </c>
@@ -4035,7 +3896,7 @@
       <c r="D36" t="s">
         <v>19</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="E36" t="s">
         <v>96</v>
       </c>
       <c r="F36" t="s">
@@ -4066,7 +3927,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>74</v>
       </c>
@@ -4079,7 +3940,7 @@
       <c r="D37" t="s">
         <v>19</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="E37" t="s">
         <v>96</v>
       </c>
       <c r="F37" t="s">
@@ -4110,7 +3971,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>74</v>
       </c>
@@ -4123,7 +3984,7 @@
       <c r="D38" t="s">
         <v>19</v>
       </c>
-      <c r="E38" s="2" t="s">
+      <c r="E38" t="s">
         <v>37</v>
       </c>
       <c r="F38" t="s">
@@ -4154,7 +4015,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>74</v>
       </c>
@@ -4167,7 +4028,7 @@
       <c r="D39" t="s">
         <v>19</v>
       </c>
-      <c r="E39" s="2" t="s">
+      <c r="E39" t="s">
         <v>37</v>
       </c>
       <c r="F39" t="s">
@@ -4198,7 +4059,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>74</v>
       </c>
@@ -4211,7 +4072,7 @@
       <c r="D40" t="s">
         <v>19</v>
       </c>
-      <c r="E40" s="2" t="s">
+      <c r="E40" t="s">
         <v>99</v>
       </c>
       <c r="F40" t="s">
@@ -4242,7 +4103,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>74</v>
       </c>
@@ -4255,7 +4116,7 @@
       <c r="D41" t="s">
         <v>19</v>
       </c>
-      <c r="E41" s="2" t="s">
+      <c r="E41" t="s">
         <v>99</v>
       </c>
       <c r="F41" t="s">
@@ -4286,7 +4147,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>75</v>
       </c>
@@ -4299,7 +4160,7 @@
       <c r="D42" t="s">
         <v>19</v>
       </c>
-      <c r="E42" s="2" t="s">
+      <c r="E42" t="s">
         <v>38</v>
       </c>
       <c r="F42" t="s">
@@ -4330,7 +4191,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>75</v>
       </c>
@@ -4343,7 +4204,7 @@
       <c r="D43" t="s">
         <v>19</v>
       </c>
-      <c r="E43" s="2" t="s">
+      <c r="E43" t="s">
         <v>38</v>
       </c>
       <c r="F43" t="s">
@@ -4374,7 +4235,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>75</v>
       </c>
@@ -4387,7 +4248,7 @@
       <c r="D44" t="s">
         <v>19</v>
       </c>
-      <c r="E44" s="2" t="s">
+      <c r="E44" t="s">
         <v>39</v>
       </c>
       <c r="F44" t="s">
@@ -4418,7 +4279,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>75</v>
       </c>
@@ -4431,7 +4292,7 @@
       <c r="D45" t="s">
         <v>19</v>
       </c>
-      <c r="E45" s="2" t="s">
+      <c r="E45" t="s">
         <v>39</v>
       </c>
       <c r="F45" t="s">
@@ -4461,150 +4322,6 @@
       <c r="N45" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="D46" s="2"/>
-    </row>
-    <row r="49" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D49" s="2"/>
-    </row>
-    <row r="50" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D50" s="2"/>
-    </row>
-    <row r="51" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D51" s="2"/>
-    </row>
-    <row r="52" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D52" s="2"/>
-    </row>
-    <row r="53" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D53" s="2"/>
-    </row>
-    <row r="54" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D54" s="2"/>
-    </row>
-    <row r="55" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D55" s="2"/>
-    </row>
-    <row r="56" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D56" s="2"/>
-    </row>
-    <row r="57" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D57" s="2"/>
-    </row>
-    <row r="58" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D58" s="2"/>
-    </row>
-    <row r="59" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D59" s="2"/>
-    </row>
-    <row r="60" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D60" s="2"/>
-    </row>
-    <row r="61" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D61" s="2"/>
-    </row>
-    <row r="62" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D62" s="2"/>
-    </row>
-    <row r="63" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D63" s="2"/>
-    </row>
-    <row r="64" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D64" s="2"/>
-    </row>
-    <row r="65" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D65" s="2"/>
-    </row>
-    <row r="66" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D66" s="2"/>
-    </row>
-    <row r="67" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D67" s="2"/>
-    </row>
-    <row r="68" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D68" s="2"/>
-    </row>
-    <row r="69" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D69" s="2"/>
-    </row>
-    <row r="70" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D70" s="2"/>
-    </row>
-    <row r="71" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D71" s="2"/>
-    </row>
-    <row r="72" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D72" s="2"/>
-    </row>
-    <row r="75" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D75" s="2"/>
-    </row>
-    <row r="76" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D76" s="2"/>
-    </row>
-    <row r="77" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D77" s="2"/>
-    </row>
-    <row r="78" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D78" s="2"/>
-    </row>
-    <row r="79" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D79" s="2"/>
-    </row>
-    <row r="80" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D80" s="2"/>
-    </row>
-    <row r="81" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D81" s="2"/>
-    </row>
-    <row r="82" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D82" s="2"/>
-    </row>
-    <row r="83" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D83" s="2"/>
-    </row>
-    <row r="84" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D84" s="2"/>
-    </row>
-    <row r="85" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D85" s="2"/>
-    </row>
-    <row r="86" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D86" s="2"/>
-    </row>
-    <row r="87" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D87" s="2"/>
-    </row>
-    <row r="88" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D88" s="2"/>
-    </row>
-    <row r="89" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D89" s="2"/>
-    </row>
-    <row r="90" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D90" s="2"/>
-    </row>
-    <row r="91" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D91" s="2"/>
-    </row>
-    <row r="92" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D92" s="2"/>
-    </row>
-    <row r="93" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D93" s="2"/>
-    </row>
-    <row r="94" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D94" s="2"/>
-    </row>
-    <row r="95" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D95" s="2"/>
-    </row>
-    <row r="96" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D96" s="2"/>
-    </row>
-    <row r="97" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D97" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4616,25 +4333,25 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F55EE6AA-34A4-4821-B841-CD8266F82E80}">
-  <dimension ref="A1:N103"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:N73"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="143.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="67.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="153.109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.5546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="50.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="56.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="51.109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="31.5546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="143.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="67.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="153.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="50.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="56.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="51.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="31.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>71</v>
       </c>
@@ -4678,7 +4395,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>65</v>
       </c>
@@ -4691,7 +4408,7 @@
       <c r="D2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" t="s">
         <v>20</v>
       </c>
       <c r="F2" t="s">
@@ -4722,7 +4439,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>65</v>
       </c>
@@ -4735,7 +4452,7 @@
       <c r="D3" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" t="s">
         <v>20</v>
       </c>
       <c r="F3" t="s">
@@ -4766,7 +4483,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>65</v>
       </c>
@@ -4810,7 +4527,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>65</v>
       </c>
@@ -4823,7 +4540,7 @@
       <c r="D5" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" t="s">
         <v>21</v>
       </c>
       <c r="F5" t="s">
@@ -4854,7 +4571,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>65</v>
       </c>
@@ -4867,7 +4584,7 @@
       <c r="D6" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" t="s">
         <v>21</v>
       </c>
       <c r="F6" t="s">
@@ -4898,7 +4615,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>65</v>
       </c>
@@ -4911,7 +4628,7 @@
       <c r="D7" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" t="s">
         <v>21</v>
       </c>
       <c r="F7" t="s">
@@ -4942,8 +4659,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
         <v>65</v>
       </c>
       <c r="B8" t="s">
@@ -4955,7 +4672,7 @@
       <c r="D8" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" t="s">
         <v>20</v>
       </c>
       <c r="F8" t="s">
@@ -4986,8 +4703,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
         <v>65</v>
       </c>
       <c r="B9" t="s">
@@ -4999,7 +4716,7 @@
       <c r="D9" t="s">
         <v>17</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" t="s">
         <v>20</v>
       </c>
       <c r="F9" t="s">
@@ -5030,7 +4747,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>73</v>
       </c>
@@ -5043,7 +4760,7 @@
       <c r="D10" t="s">
         <v>18</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" t="s">
         <v>22</v>
       </c>
       <c r="F10" t="s">
@@ -5074,7 +4791,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>73</v>
       </c>
@@ -5087,7 +4804,7 @@
       <c r="D11" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" t="s">
         <v>22</v>
       </c>
       <c r="F11" t="s">
@@ -5118,7 +4835,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>73</v>
       </c>
@@ -5131,7 +4848,7 @@
       <c r="D12" t="s">
         <v>18</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" t="s">
         <v>23</v>
       </c>
       <c r="F12" t="s">
@@ -5162,7 +4879,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>73</v>
       </c>
@@ -5175,7 +4892,7 @@
       <c r="D13" t="s">
         <v>18</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" t="s">
         <v>23</v>
       </c>
       <c r="F13" t="s">
@@ -5206,7 +4923,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>73</v>
       </c>
@@ -5219,7 +4936,7 @@
       <c r="D14" t="s">
         <v>19</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" t="s">
         <v>81</v>
       </c>
       <c r="F14" t="s">
@@ -5250,7 +4967,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>73</v>
       </c>
@@ -5263,7 +4980,7 @@
       <c r="D15" t="s">
         <v>19</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" t="s">
         <v>81</v>
       </c>
       <c r="F15" t="s">
@@ -5294,7 +5011,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>73</v>
       </c>
@@ -5307,7 +5024,7 @@
       <c r="D16" t="s">
         <v>19</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" t="s">
         <v>88</v>
       </c>
       <c r="F16" t="s">
@@ -5338,7 +5055,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>73</v>
       </c>
@@ -5351,7 +5068,7 @@
       <c r="D17" t="s">
         <v>19</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" t="s">
         <v>88</v>
       </c>
       <c r="F17" t="s">
@@ -5382,7 +5099,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>73</v>
       </c>
@@ -5395,7 +5112,7 @@
       <c r="D18" t="s">
         <v>19</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" t="s">
         <v>85</v>
       </c>
       <c r="F18" t="s">
@@ -5426,7 +5143,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>73</v>
       </c>
@@ -5439,7 +5156,7 @@
       <c r="D19" t="s">
         <v>19</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" t="s">
         <v>85</v>
       </c>
       <c r="F19" t="s">
@@ -5470,7 +5187,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>73</v>
       </c>
@@ -5483,7 +5200,7 @@
       <c r="D20" t="s">
         <v>19</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" t="s">
         <v>24</v>
       </c>
       <c r="F20" t="s">
@@ -5514,7 +5231,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>73</v>
       </c>
@@ -5527,7 +5244,7 @@
       <c r="D21" t="s">
         <v>19</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" t="s">
         <v>24</v>
       </c>
       <c r="F21" t="s">
@@ -5558,7 +5275,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>74</v>
       </c>
@@ -5571,7 +5288,7 @@
       <c r="D22" t="s">
         <v>19</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" t="s">
         <v>25</v>
       </c>
       <c r="F22" t="s">
@@ -5602,7 +5319,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>74</v>
       </c>
@@ -5615,7 +5332,7 @@
       <c r="D23" t="s">
         <v>19</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="E23" t="s">
         <v>25</v>
       </c>
       <c r="F23" t="s">
@@ -5646,7 +5363,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>76</v>
       </c>
@@ -5659,7 +5376,7 @@
       <c r="D24" t="s">
         <v>19</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="E24" t="s">
         <v>29</v>
       </c>
       <c r="F24" t="s">
@@ -5690,7 +5407,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>76</v>
       </c>
@@ -5703,7 +5420,7 @@
       <c r="D25" t="s">
         <v>19</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="E25" t="s">
         <v>29</v>
       </c>
       <c r="F25" t="s">
@@ -5734,7 +5451,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>76</v>
       </c>
@@ -5747,7 +5464,7 @@
       <c r="D26" t="s">
         <v>19</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" t="s">
         <v>31</v>
       </c>
       <c r="F26" t="s">
@@ -5778,7 +5495,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>76</v>
       </c>
@@ -5791,7 +5508,7 @@
       <c r="D27" t="s">
         <v>19</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" t="s">
         <v>31</v>
       </c>
       <c r="F27" t="s">
@@ -5822,7 +5539,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>76</v>
       </c>
@@ -5832,10 +5549,10 @@
       <c r="C28" t="s">
         <v>4</v>
       </c>
-      <c r="D28" s="3" t="s">
+      <c r="D28" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E28" s="2" t="s">
+      <c r="E28" t="s">
         <v>102</v>
       </c>
       <c r="F28" t="s">
@@ -5866,7 +5583,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>76</v>
       </c>
@@ -5876,10 +5593,10 @@
       <c r="C29" t="s">
         <v>4</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E29" s="2" t="s">
+      <c r="E29" t="s">
         <v>102</v>
       </c>
       <c r="F29" t="s">
@@ -5910,7 +5627,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>76</v>
       </c>
@@ -5920,10 +5637,10 @@
       <c r="C30" t="s">
         <v>4</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="E30" t="s">
         <v>105</v>
       </c>
       <c r="F30" t="s">
@@ -5954,7 +5671,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>76</v>
       </c>
@@ -5964,10 +5681,10 @@
       <c r="C31" t="s">
         <v>4</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E31" s="2" t="s">
+      <c r="E31" t="s">
         <v>105</v>
       </c>
       <c r="F31" t="s">
@@ -5998,7 +5715,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>76</v>
       </c>
@@ -6008,10 +5725,10 @@
       <c r="C32" t="s">
         <v>4</v>
       </c>
-      <c r="D32" s="3" t="s">
+      <c r="D32" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E32" s="2" t="s">
+      <c r="E32" t="s">
         <v>108</v>
       </c>
       <c r="F32" t="s">
@@ -6042,7 +5759,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>76</v>
       </c>
@@ -6052,10 +5769,10 @@
       <c r="C33" t="s">
         <v>4</v>
       </c>
-      <c r="D33" s="3" t="s">
+      <c r="D33" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="E33" t="s">
         <v>108</v>
       </c>
       <c r="F33" t="s">
@@ -6086,7 +5803,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>74</v>
       </c>
@@ -6099,7 +5816,7 @@
       <c r="D34" t="s">
         <v>19</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="E34" t="s">
         <v>34</v>
       </c>
       <c r="F34" t="s">
@@ -6130,7 +5847,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>74</v>
       </c>
@@ -6143,7 +5860,7 @@
       <c r="D35" t="s">
         <v>19</v>
       </c>
-      <c r="E35" s="2" t="s">
+      <c r="E35" t="s">
         <v>34</v>
       </c>
       <c r="F35" t="s">
@@ -6174,7 +5891,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>74</v>
       </c>
@@ -6187,7 +5904,7 @@
       <c r="D36" t="s">
         <v>19</v>
       </c>
-      <c r="E36" s="2" t="s">
+      <c r="E36" t="s">
         <v>93</v>
       </c>
       <c r="F36" t="s">
@@ -6218,7 +5935,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>74</v>
       </c>
@@ -6231,7 +5948,7 @@
       <c r="D37" t="s">
         <v>19</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="E37" t="s">
         <v>93</v>
       </c>
       <c r="F37" t="s">
@@ -6262,7 +5979,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>74</v>
       </c>
@@ -6275,7 +5992,7 @@
       <c r="D38" t="s">
         <v>19</v>
       </c>
-      <c r="E38" s="2" t="s">
+      <c r="E38" t="s">
         <v>96</v>
       </c>
       <c r="F38" t="s">
@@ -6306,7 +6023,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>74</v>
       </c>
@@ -6319,7 +6036,7 @@
       <c r="D39" t="s">
         <v>19</v>
       </c>
-      <c r="E39" s="2" t="s">
+      <c r="E39" t="s">
         <v>96</v>
       </c>
       <c r="F39" t="s">
@@ -6350,7 +6067,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>74</v>
       </c>
@@ -6363,7 +6080,7 @@
       <c r="D40" t="s">
         <v>19</v>
       </c>
-      <c r="E40" s="2" t="s">
+      <c r="E40" t="s">
         <v>37</v>
       </c>
       <c r="F40" t="s">
@@ -6394,7 +6111,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>74</v>
       </c>
@@ -6407,7 +6124,7 @@
       <c r="D41" t="s">
         <v>19</v>
       </c>
-      <c r="E41" s="2" t="s">
+      <c r="E41" t="s">
         <v>37</v>
       </c>
       <c r="F41" t="s">
@@ -6438,7 +6155,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>74</v>
       </c>
@@ -6451,7 +6168,7 @@
       <c r="D42" t="s">
         <v>19</v>
       </c>
-      <c r="E42" s="2" t="s">
+      <c r="E42" t="s">
         <v>99</v>
       </c>
       <c r="F42" t="s">
@@ -6482,7 +6199,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="43" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>74</v>
       </c>
@@ -6495,7 +6212,7 @@
       <c r="D43" t="s">
         <v>19</v>
       </c>
-      <c r="E43" s="2" t="s">
+      <c r="E43" t="s">
         <v>99</v>
       </c>
       <c r="F43" t="s">
@@ -6526,7 +6243,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="44" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>111</v>
       </c>
@@ -6539,7 +6256,7 @@
       <c r="D44" t="s">
         <v>19</v>
       </c>
-      <c r="E44" s="2" t="s">
+      <c r="E44" t="s">
         <v>38</v>
       </c>
       <c r="F44" t="s">
@@ -6570,7 +6287,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="45" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>111</v>
       </c>
@@ -6583,7 +6300,7 @@
       <c r="D45" t="s">
         <v>19</v>
       </c>
-      <c r="E45" s="2" t="s">
+      <c r="E45" t="s">
         <v>38</v>
       </c>
       <c r="F45" t="s">
@@ -6614,7 +6331,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="46" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>111</v>
       </c>
@@ -6627,7 +6344,7 @@
       <c r="D46" t="s">
         <v>19</v>
       </c>
-      <c r="E46" s="2" t="s">
+      <c r="E46" t="s">
         <v>39</v>
       </c>
       <c r="F46" t="s">
@@ -6658,7 +6375,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="47" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>111</v>
       </c>
@@ -6671,7 +6388,7 @@
       <c r="D47" t="s">
         <v>19</v>
       </c>
-      <c r="E47" s="2" t="s">
+      <c r="E47" t="s">
         <v>39</v>
       </c>
       <c r="F47" t="s">
@@ -6702,8 +6419,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="48" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A48" s="3" t="s">
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
         <v>111</v>
       </c>
       <c r="B48" t="s">
@@ -6715,7 +6432,7 @@
       <c r="D48" t="s">
         <v>150</v>
       </c>
-      <c r="E48" s="2" t="s">
+      <c r="E48" t="s">
         <v>152</v>
       </c>
       <c r="F48" t="s">
@@ -6746,8 +6463,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="49" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A49" s="3" t="s">
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
         <v>111</v>
       </c>
       <c r="B49" t="s">
@@ -6759,7 +6476,7 @@
       <c r="D49" t="s">
         <v>150</v>
       </c>
-      <c r="E49" s="2" t="s">
+      <c r="E49" t="s">
         <v>152</v>
       </c>
       <c r="F49" t="s">
@@ -6790,8 +6507,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="50" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A50" s="3" t="s">
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
         <v>111</v>
       </c>
       <c r="B50" t="s">
@@ -6803,7 +6520,7 @@
       <c r="D50" t="s">
         <v>150</v>
       </c>
-      <c r="E50" s="2" t="s">
+      <c r="E50" t="s">
         <v>153</v>
       </c>
       <c r="F50" t="s">
@@ -6834,8 +6551,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="51" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A51" s="3" t="s">
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
         <v>111</v>
       </c>
       <c r="B51" t="s">
@@ -6847,7 +6564,7 @@
       <c r="D51" t="s">
         <v>150</v>
       </c>
-      <c r="E51" s="2" t="s">
+      <c r="E51" t="s">
         <v>153</v>
       </c>
       <c r="F51" t="s">
@@ -6878,8 +6595,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="52" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A52" s="3" t="s">
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
         <v>111</v>
       </c>
       <c r="B52" t="s">
@@ -6891,7 +6608,7 @@
       <c r="D52" t="s">
         <v>150</v>
       </c>
-      <c r="E52" s="2" t="s">
+      <c r="E52" t="s">
         <v>154</v>
       </c>
       <c r="F52" t="s">
@@ -6922,8 +6639,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="53" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A53" s="3" t="s">
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="s">
         <v>111</v>
       </c>
       <c r="B53" t="s">
@@ -6935,7 +6652,7 @@
       <c r="D53" t="s">
         <v>150</v>
       </c>
-      <c r="E53" s="2" t="s">
+      <c r="E53" t="s">
         <v>154</v>
       </c>
       <c r="F53" t="s">
@@ -6966,8 +6683,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="54" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A54" s="3" t="s">
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
         <v>111</v>
       </c>
       <c r="B54" t="s">
@@ -6979,7 +6696,7 @@
       <c r="D54" t="s">
         <v>150</v>
       </c>
-      <c r="E54" s="2" t="s">
+      <c r="E54" t="s">
         <v>189</v>
       </c>
       <c r="F54" t="s">
@@ -7010,8 +6727,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="55" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A55" s="3" t="s">
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="s">
         <v>111</v>
       </c>
       <c r="B55" t="s">
@@ -7023,7 +6740,7 @@
       <c r="D55" t="s">
         <v>150</v>
       </c>
-      <c r="E55" s="2" t="s">
+      <c r="E55" t="s">
         <v>189</v>
       </c>
       <c r="F55" t="s">
@@ -7054,8 +6771,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="56" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A56" s="4" t="s">
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A56" s="3" t="s">
         <v>111</v>
       </c>
       <c r="B56" t="s">
@@ -7067,7 +6784,7 @@
       <c r="D56" t="s">
         <v>151</v>
       </c>
-      <c r="E56" s="2" t="s">
+      <c r="E56" t="s">
         <v>155</v>
       </c>
       <c r="F56" t="s">
@@ -7098,8 +6815,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="57" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A57" s="4" t="s">
+    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A57" s="3" t="s">
         <v>111</v>
       </c>
       <c r="B57" t="s">
@@ -7111,7 +6828,7 @@
       <c r="D57" t="s">
         <v>151</v>
       </c>
-      <c r="E57" s="2" t="s">
+      <c r="E57" t="s">
         <v>155</v>
       </c>
       <c r="F57" t="s">
@@ -7142,8 +6859,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="58" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A58" s="4" t="s">
+    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A58" s="3" t="s">
         <v>111</v>
       </c>
       <c r="B58" t="s">
@@ -7155,7 +6872,7 @@
       <c r="D58" t="s">
         <v>151</v>
       </c>
-      <c r="E58" s="2" t="s">
+      <c r="E58" t="s">
         <v>192</v>
       </c>
       <c r="F58" t="s">
@@ -7186,8 +6903,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="59" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A59" s="4" t="s">
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A59" s="3" t="s">
         <v>111</v>
       </c>
       <c r="B59" t="s">
@@ -7199,7 +6916,7 @@
       <c r="D59" t="s">
         <v>151</v>
       </c>
-      <c r="E59" s="2" t="s">
+      <c r="E59" t="s">
         <v>192</v>
       </c>
       <c r="F59" t="s">
@@ -7230,8 +6947,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="60" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A60" s="4" t="s">
+    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A60" s="3" t="s">
         <v>111</v>
       </c>
       <c r="B60" t="s">
@@ -7243,7 +6960,7 @@
       <c r="D60" t="s">
         <v>151</v>
       </c>
-      <c r="E60" s="2" t="s">
+      <c r="E60" t="s">
         <v>158</v>
       </c>
       <c r="F60" t="s">
@@ -7274,8 +6991,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="61" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A61" s="4" t="s">
+    <row r="61" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A61" s="3" t="s">
         <v>111</v>
       </c>
       <c r="B61" t="s">
@@ -7287,7 +7004,7 @@
       <c r="D61" t="s">
         <v>151</v>
       </c>
-      <c r="E61" s="2" t="s">
+      <c r="E61" t="s">
         <v>158</v>
       </c>
       <c r="F61" t="s">
@@ -7318,8 +7035,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="62" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A62" s="3" t="s">
+    <row r="62" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A62" s="2" t="s">
         <v>161</v>
       </c>
       <c r="B62" t="s">
@@ -7331,7 +7048,7 @@
       <c r="D62" t="s">
         <v>19</v>
       </c>
-      <c r="E62" s="2" t="s">
+      <c r="E62" t="s">
         <v>195</v>
       </c>
       <c r="F62" t="s">
@@ -7362,8 +7079,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="63" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A63" s="3" t="s">
+    <row r="63" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A63" s="2" t="s">
         <v>161</v>
       </c>
       <c r="B63" t="s">
@@ -7375,7 +7092,7 @@
       <c r="D63" t="s">
         <v>19</v>
       </c>
-      <c r="E63" s="2" t="s">
+      <c r="E63" t="s">
         <v>195</v>
       </c>
       <c r="F63" t="s">
@@ -7406,8 +7123,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="64" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A64" s="3" t="s">
+    <row r="64" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A64" s="2" t="s">
         <v>161</v>
       </c>
       <c r="B64" t="s">
@@ -7419,7 +7136,7 @@
       <c r="D64" t="s">
         <v>19</v>
       </c>
-      <c r="E64" s="2" t="s">
+      <c r="E64" t="s">
         <v>196</v>
       </c>
       <c r="F64" t="s">
@@ -7450,8 +7167,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="65" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A65" s="3" t="s">
+    <row r="65" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A65" s="2" t="s">
         <v>161</v>
       </c>
       <c r="B65" t="s">
@@ -7463,7 +7180,7 @@
       <c r="D65" t="s">
         <v>19</v>
       </c>
-      <c r="E65" s="2" t="s">
+      <c r="E65" t="s">
         <v>196</v>
       </c>
       <c r="F65" t="s">
@@ -7494,8 +7211,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="66" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A66" s="3" t="s">
+    <row r="66" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A66" s="2" t="s">
         <v>161</v>
       </c>
       <c r="B66" t="s">
@@ -7507,7 +7224,7 @@
       <c r="D66" t="s">
         <v>19</v>
       </c>
-      <c r="E66" s="2" t="s">
+      <c r="E66" t="s">
         <v>197</v>
       </c>
       <c r="F66" t="s">
@@ -7538,8 +7255,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A67" s="3" t="s">
+    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A67" s="2" t="s">
         <v>161</v>
       </c>
       <c r="B67" t="s">
@@ -7551,7 +7268,7 @@
       <c r="D67" t="s">
         <v>19</v>
       </c>
-      <c r="E67" s="2" t="s">
+      <c r="E67" t="s">
         <v>197</v>
       </c>
       <c r="F67" t="s">
@@ -7582,8 +7299,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="68" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A68" s="3" t="s">
+    <row r="68" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A68" s="2" t="s">
         <v>161</v>
       </c>
       <c r="B68" t="s">
@@ -7595,7 +7312,7 @@
       <c r="D68" t="s">
         <v>19</v>
       </c>
-      <c r="E68" s="2" t="s">
+      <c r="E68" t="s">
         <v>198</v>
       </c>
       <c r="F68" t="s">
@@ -7626,8 +7343,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="69" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A69" s="3" t="s">
+    <row r="69" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A69" s="2" t="s">
         <v>161</v>
       </c>
       <c r="B69" t="s">
@@ -7639,7 +7356,7 @@
       <c r="D69" t="s">
         <v>19</v>
       </c>
-      <c r="E69" s="2" t="s">
+      <c r="E69" t="s">
         <v>198</v>
       </c>
       <c r="F69" t="s">
@@ -7670,8 +7387,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="70" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A70" s="3" t="s">
+    <row r="70" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A70" s="2" t="s">
         <v>161</v>
       </c>
       <c r="B70" t="s">
@@ -7683,7 +7400,7 @@
       <c r="D70" t="s">
         <v>19</v>
       </c>
-      <c r="E70" s="2" t="s">
+      <c r="E70" t="s">
         <v>199</v>
       </c>
       <c r="F70" t="s">
@@ -7714,8 +7431,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="71" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A71" s="3" t="s">
+    <row r="71" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A71" s="2" t="s">
         <v>161</v>
       </c>
       <c r="B71" t="s">
@@ -7727,7 +7444,7 @@
       <c r="D71" t="s">
         <v>19</v>
       </c>
-      <c r="E71" s="2" t="s">
+      <c r="E71" t="s">
         <v>199</v>
       </c>
       <c r="F71" t="s">
@@ -7758,8 +7475,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="72" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A72" s="3" t="s">
+    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A72" s="2" t="s">
         <v>161</v>
       </c>
       <c r="B72" t="s">
@@ -7771,7 +7488,7 @@
       <c r="D72" t="s">
         <v>19</v>
       </c>
-      <c r="E72" s="2" t="s">
+      <c r="E72" t="s">
         <v>200</v>
       </c>
       <c r="F72" t="s">
@@ -7802,8 +7519,8 @@
         <v>64</v>
       </c>
     </row>
-    <row r="73" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A73" s="3" t="s">
+    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A73" s="2" t="s">
         <v>161</v>
       </c>
       <c r="B73" t="s">
@@ -7815,7 +7532,7 @@
       <c r="D73" t="s">
         <v>19</v>
       </c>
-      <c r="E73" s="2" t="s">
+      <c r="E73" t="s">
         <v>200</v>
       </c>
       <c r="F73" t="s">
@@ -7845,90 +7562,6 @@
       <c r="N73" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="74" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="D74" s="2"/>
-    </row>
-    <row r="75" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="D75" s="2"/>
-    </row>
-    <row r="76" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="D76" s="2"/>
-    </row>
-    <row r="77" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="D77" s="2"/>
-    </row>
-    <row r="78" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="D78" s="2"/>
-    </row>
-    <row r="81" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D81" s="2"/>
-    </row>
-    <row r="82" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D82" s="2"/>
-    </row>
-    <row r="83" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D83" s="2"/>
-    </row>
-    <row r="84" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D84" s="2"/>
-    </row>
-    <row r="85" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D85" s="2"/>
-    </row>
-    <row r="86" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D86" s="2"/>
-    </row>
-    <row r="87" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D87" s="2"/>
-    </row>
-    <row r="88" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D88" s="2"/>
-    </row>
-    <row r="89" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D89" s="2"/>
-    </row>
-    <row r="90" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D90" s="2"/>
-    </row>
-    <row r="91" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D91" s="2"/>
-    </row>
-    <row r="92" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D92" s="2"/>
-    </row>
-    <row r="93" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D93" s="2"/>
-    </row>
-    <row r="94" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D94" s="2"/>
-    </row>
-    <row r="95" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D95" s="2"/>
-    </row>
-    <row r="96" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D96" s="2"/>
-    </row>
-    <row r="97" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D97" s="2"/>
-    </row>
-    <row r="98" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D98" s="2"/>
-    </row>
-    <row r="99" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D99" s="2"/>
-    </row>
-    <row r="100" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D100" s="2"/>
-    </row>
-    <row r="101" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D101" s="2"/>
-    </row>
-    <row r="102" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D102" s="2"/>
-    </row>
-    <row r="103" spans="4:4" x14ac:dyDescent="0.3">
-      <c r="D103" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>